<commit_message>
Update data files - Bot run at 2026-09-14 00:41:12 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="L2" t="n">
-        <v>0.001046</v>
+        <v>0.001036</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-09T05:55:08.246990</t>
+          <t>2026-09-14T00:41:01.591307</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>465</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00465</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-09T05:55:08.246990</t>
+          <t>2026-09-14T00:41:01.591307</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-09T05:55:08.246990</t>
+          <t>2026-09-14T00:41:01.591307</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-09T05:55:08.246990</t>
+          <t>2026-09-14T00:41:01.591307</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-09T05:55:08.246990</t>
+          <t>2026-09-14T00:41:01.591307</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-09T05:55:08.246990</t>
+          <t>2026-09-14T00:41:01.591307</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-09T05:55:08.246990</t>
+          <t>2026-09-14T00:41:01.591307</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-09T05:55:08.246990</t>
+          <t>2026-09-14T00:41:01.591307</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-09T05:55:08.246990</t>
+          <t>2026-09-14T00:41:01.591307</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-09T05:55:08.246990</t>
+          <t>2026-09-14T00:41:01.591307</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-09T05:55:08.246990</t>
+          <t>2026-09-14T00:41:01.591307</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-09T05:55:08.246990</t>
+          <t>2026-09-14T00:41:01.591307</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-09T05:55:08.246990</t>
+          <t>2026-09-14T00:41:01.591307</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-14 05:45:10 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>1047</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.01047</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-18 14:23:13 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>518</v>
+        <v>467</v>
       </c>
       <c r="L2" t="n">
-        <v>0.001036</v>
+        <v>0.000934</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:01.591307</t>
+          <t>2026-09-18T14:23:09.978538</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>1047</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.01047</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:01.591307</t>
+          <t>2026-09-18T14:23:09.978538</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:01.591307</t>
+          <t>2026-09-18T14:23:09.978538</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:01.591307</t>
+          <t>2026-09-18T14:23:09.978538</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:01.591307</t>
+          <t>2026-09-18T14:23:09.978538</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:01.591307</t>
+          <t>2026-09-18T14:23:09.978538</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:01.591307</t>
+          <t>2026-09-18T14:23:09.978538</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:01.591307</t>
+          <t>2026-09-18T14:23:09.978538</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:01.591307</t>
+          <t>2026-09-18T14:23:09.978538</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:01.591307</t>
+          <t>2026-09-18T14:23:09.978538</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:01.591307</t>
+          <t>2026-09-18T14:23:09.978538</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:01.591307</t>
+          <t>2026-09-18T14:23:09.978538</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-14T00:41:01.591307</t>
+          <t>2026-09-18T14:23:09.978538</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-26 01:10:49 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>467</v>
+        <v>502</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000934</v>
+        <v>0.001004</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-18T14:23:09.978538</t>
+          <t>2026-09-26T01:10:43.590181</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-18T14:23:09.978538</t>
+          <t>2026-09-26T01:10:43.590181</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-18T14:23:09.978538</t>
+          <t>2026-09-26T01:10:43.590181</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-18T14:23:09.978538</t>
+          <t>2026-09-26T01:10:43.590181</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-18T14:23:09.978538</t>
+          <t>2026-09-26T01:10:43.590181</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-18T14:23:09.978538</t>
+          <t>2026-09-26T01:10:43.590181</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-18T14:23:09.978538</t>
+          <t>2026-09-26T01:10:43.590181</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-18T14:23:09.978538</t>
+          <t>2026-09-26T01:10:43.590181</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-18T14:23:09.978538</t>
+          <t>2026-09-26T01:10:43.590181</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-18T14:23:09.978538</t>
+          <t>2026-09-26T01:10:43.590181</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-18T14:23:09.978538</t>
+          <t>2026-09-26T01:10:43.590181</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-18T14:23:09.978538</t>
+          <t>2026-09-26T01:10:43.590181</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-18T14:23:09.978538</t>
+          <t>2026-09-26T01:10:43.590181</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-28 01:07:42 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>502</v>
+        <v>483</v>
       </c>
       <c r="L2" t="n">
-        <v>0.001004</v>
+        <v>0.000966</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-26T01:10:43.590181</t>
+          <t>2026-09-28T01:07:33.501954</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-26T01:10:43.590181</t>
+          <t>2026-09-28T01:07:33.501954</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-26T01:10:43.590181</t>
+          <t>2026-09-28T01:07:33.501954</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-26T01:10:43.590181</t>
+          <t>2026-09-28T01:07:33.501954</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-26T01:10:43.590181</t>
+          <t>2026-09-28T01:07:33.501954</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-26T01:10:43.590181</t>
+          <t>2026-09-28T01:07:33.501954</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-26T01:10:43.590181</t>
+          <t>2026-09-28T01:07:33.501954</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-26T01:10:43.590181</t>
+          <t>2026-09-28T01:07:33.501954</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-26T01:10:43.590181</t>
+          <t>2026-09-28T01:07:33.501954</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-26T01:10:43.590181</t>
+          <t>2026-09-28T01:07:33.501954</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-26T01:10:43.590181</t>
+          <t>2026-09-28T01:07:33.501954</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-26T01:10:43.590181</t>
+          <t>2026-09-28T01:07:33.501954</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-26T01:10:43.590181</t>
+          <t>2026-09-28T01:07:33.501954</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-09-29 01:28:01 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>483</v>
+        <v>472</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000966</v>
+        <v>0.000944</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-28T01:07:33.501954</t>
+          <t>2026-09-29T01:27:57.545946</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-28T01:07:33.501954</t>
+          <t>2026-09-29T01:27:57.545946</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-28T01:07:33.501954</t>
+          <t>2026-09-29T01:27:57.545946</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-28T01:07:33.501954</t>
+          <t>2026-09-29T01:27:57.545946</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-28T01:07:33.501954</t>
+          <t>2026-09-29T01:27:57.545946</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-28T01:07:33.501954</t>
+          <t>2026-09-29T01:27:57.545946</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-28T01:07:33.501954</t>
+          <t>2026-09-29T01:27:57.545946</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-28T01:07:33.501954</t>
+          <t>2026-09-29T01:27:57.545946</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-28T01:07:33.501954</t>
+          <t>2026-09-29T01:27:57.545946</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-28T01:07:33.501954</t>
+          <t>2026-09-29T01:27:57.545946</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-28T01:07:33.501954</t>
+          <t>2026-09-29T01:27:57.545946</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-28T01:07:33.501954</t>
+          <t>2026-09-29T01:27:57.545946</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-28T01:07:33.501954</t>
+          <t>2026-09-29T01:27:57.545946</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-03 14:34:21 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="L2" t="n">
-        <v>0.000944</v>
+        <v>0.0009300000000000001</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:57.545946</t>
+          <t>2026-10-03T14:34:13.936111</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.0048</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:57.545946</t>
+          <t>2026-10-03T14:34:13.936111</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:57.545946</t>
+          <t>2026-10-03T14:34:13.936111</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:57.545946</t>
+          <t>2026-10-03T14:34:13.936111</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:57.545946</t>
+          <t>2026-10-03T14:34:13.936111</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:57.545946</t>
+          <t>2026-10-03T14:34:13.936111</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:57.545946</t>
+          <t>2026-10-03T14:34:13.936111</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:57.545946</t>
+          <t>2026-10-03T14:34:13.936111</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:57.545946</t>
+          <t>2026-10-03T14:34:13.936111</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:57.545946</t>
+          <t>2026-10-03T14:34:13.936111</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:57.545946</t>
+          <t>2026-10-03T14:34:13.936111</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:57.545946</t>
+          <t>2026-10-03T14:34:13.936111</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-29T01:27:57.545946</t>
+          <t>2026-10-03T14:34:13.936111</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-14 14:20:06 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>465</v>
+        <v>495</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0009300000000000001</v>
+        <v>0.00099</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-03T14:34:13.936111</t>
+          <t>2026-10-14T14:20:03.129257</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>480</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0048</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-03T14:34:13.936111</t>
+          <t>2026-10-14T14:20:03.129257</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-03T14:34:13.936111</t>
+          <t>2026-10-14T14:20:03.129257</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-03T14:34:13.936111</t>
+          <t>2026-10-14T14:20:03.129257</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-03T14:34:13.936111</t>
+          <t>2026-10-14T14:20:03.129257</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-03T14:34:13.936111</t>
+          <t>2026-10-14T14:20:03.129257</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-03T14:34:13.936111</t>
+          <t>2026-10-14T14:20:03.129257</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-03T14:34:13.936111</t>
+          <t>2026-10-14T14:20:03.129257</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-03T14:34:13.936111</t>
+          <t>2026-10-14T14:20:03.129257</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-03T14:34:13.936111</t>
+          <t>2026-10-14T14:20:03.129257</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-03T14:34:13.936111</t>
+          <t>2026-10-14T14:20:03.129257</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-03T14:34:13.936111</t>
+          <t>2026-10-14T14:20:03.129257</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-03T14:34:13.936111</t>
+          <t>2026-10-14T14:20:03.129257</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-15 00:44:21 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>502</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00502</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-16 05:40:16 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="L2" t="n">
-        <v>0.00099</v>
+        <v>0.001</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-14T14:20:03.129257</t>
+          <t>2026-10-16T05:40:10.635506</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>502</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00502</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-14T14:20:03.129257</t>
+          <t>2026-10-16T05:40:10.635506</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-14T14:20:03.129257</t>
+          <t>2026-10-16T05:40:10.635506</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-14T14:20:03.129257</t>
+          <t>2026-10-16T05:40:10.635506</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-14T14:20:03.129257</t>
+          <t>2026-10-16T05:40:10.635506</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-14T14:20:03.129257</t>
+          <t>2026-10-16T05:40:10.635506</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-14T14:20:03.129257</t>
+          <t>2026-10-16T05:40:10.635506</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-14T14:20:03.129257</t>
+          <t>2026-10-16T05:40:10.635506</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-14T14:20:03.129257</t>
+          <t>2026-10-16T05:40:10.635506</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-14T14:20:03.129257</t>
+          <t>2026-10-16T05:40:10.635506</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-14T14:20:03.129257</t>
+          <t>2026-10-16T05:40:10.635506</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-14T14:20:03.129257</t>
+          <t>2026-10-16T05:40:10.635506</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-14T14:20:03.129257</t>
+          <t>2026-10-16T05:40:10.635506</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-19 00:46:53 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>500</v>
+        <v>587</v>
       </c>
       <c r="L2" t="n">
-        <v>0.001</v>
+        <v>0.001174</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-16T05:40:10.635506</t>
+          <t>2026-10-19T00:46:44.355824</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-16T05:40:10.635506</t>
+          <t>2026-10-19T00:46:44.355824</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-16T05:40:10.635506</t>
+          <t>2026-10-19T00:46:44.355824</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-16T05:40:10.635506</t>
+          <t>2026-10-19T00:46:44.355824</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-16T05:40:10.635506</t>
+          <t>2026-10-19T00:46:44.355824</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-16T05:40:10.635506</t>
+          <t>2026-10-19T00:46:44.355824</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-16T05:40:10.635506</t>
+          <t>2026-10-19T00:46:44.355824</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-16T05:40:10.635506</t>
+          <t>2026-10-19T00:46:44.355824</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-16T05:40:10.635506</t>
+          <t>2026-10-19T00:46:44.355824</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-16T05:40:10.635506</t>
+          <t>2026-10-19T00:46:44.355824</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-16T05:40:10.635506</t>
+          <t>2026-10-19T00:46:44.355824</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-16T05:40:10.635506</t>
+          <t>2026-10-19T00:46:44.355824</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-16T05:40:10.635506</t>
+          <t>2026-10-19T00:46:44.355824</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-19 05:41:31 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -580,16 +580,16 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>568</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00568</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-21 01:51:12 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>587</v>
+        <v>521</v>
       </c>
       <c r="L2" t="n">
-        <v>0.001174</v>
+        <v>0.001042</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:44.355824</t>
+          <t>2026-10-21T01:51:03.976662</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>568</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.00568</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:44.355824</t>
+          <t>2026-10-21T01:51:03.976662</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:44.355824</t>
+          <t>2026-10-21T01:51:03.976662</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:44.355824</t>
+          <t>2026-10-21T01:51:03.976662</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:44.355824</t>
+          <t>2026-10-21T01:51:03.976662</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:44.355824</t>
+          <t>2026-10-21T01:51:03.976662</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:44.355824</t>
+          <t>2026-10-21T01:51:03.976662</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:44.355824</t>
+          <t>2026-10-21T01:51:03.976662</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:44.355824</t>
+          <t>2026-10-21T01:51:03.976662</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:44.355824</t>
+          <t>2026-10-21T01:51:03.976662</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:44.355824</t>
+          <t>2026-10-21T01:51:03.976662</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:44.355824</t>
+          <t>2026-10-21T01:51:03.976662</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-19T00:46:44.355824</t>
+          <t>2026-10-21T01:51:03.976662</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-25 13:19:22 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -535,14 +535,14 @@
         <v>6.944444444444444e-05</v>
       </c>
       <c r="K2" t="n">
-        <v>521</v>
+        <v>487</v>
       </c>
       <c r="L2" t="n">
-        <v>0.001042</v>
+        <v>0.000974</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:03.976662</t>
+          <t>2026-10-25T13:19:13.303632</t>
         </is>
       </c>
     </row>
@@ -580,20 +580,20 @@
         <v>100000</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>487</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.00487</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:03.976662</t>
+          <t>2026-10-25T13:19:13.303632</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:03.976662</t>
+          <t>2026-10-25T13:19:13.303632</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:03.976662</t>
+          <t>2026-10-25T13:19:13.303632</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:03.976662</t>
+          <t>2026-10-25T13:19:13.303632</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:03.976662</t>
+          <t>2026-10-25T13:19:13.303632</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:03.976662</t>
+          <t>2026-10-25T13:19:13.303632</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:03.976662</t>
+          <t>2026-10-25T13:19:13.303632</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:03.976662</t>
+          <t>2026-10-25T13:19:13.303632</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:03.976662</t>
+          <t>2026-10-25T13:19:13.303632</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:03.976662</t>
+          <t>2026-10-25T13:19:13.303632</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:03.976662</t>
+          <t>2026-10-25T13:19:13.303632</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-21T01:51:03.976662</t>
+          <t>2026-10-25T13:19:13.303632</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-10-26 05:46:00 UTC
</commit_message>
<xml_diff>
--- a/Free_API_Load_balancer/Limits.xlsx
+++ b/Free_API_Load_balancer/Limits.xlsx
@@ -631,16 +631,16 @@
         <v>500000</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>484</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.000968</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>

</xml_diff>